<commit_message>
relocated second stage to script; images
</commit_message>
<xml_diff>
--- a/regression_analysis/outputs_retention/second_stage_beta_regression.xlsx
+++ b/regression_analysis/outputs_retention/second_stage_beta_regression.xlsx
@@ -546,35 +546,35 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.0350807739986397</v>
+        <v>0.0536900847770649</v>
       </c>
       <c r="E2" t="n">
-        <v>3.508077399863974</v>
+        <v>5.369008477706495</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0365040756474625</v>
+        <v>0.0343616871945656</v>
       </c>
       <c r="G2" t="n">
-        <v>3.650407564746251</v>
+        <v>3.436168719456563</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3365472464058332</v>
+        <v>0.1181705984218483</v>
       </c>
       <c r="I2" t="n">
-        <v>-3.646589955931244</v>
+        <v>-1.365758457231486</v>
       </c>
       <c r="J2" t="n">
-        <v>10.66274475565919</v>
+        <v>12.10377541264447</v>
       </c>
       <c r="K2" t="n">
-        <v>930</v>
+        <v>693</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1267033639941635</v>
+        <v>0.2221208994341836</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>weight_t</t>
+          <t>earnwt_t</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -583,10 +583,10 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>0.0350807739986397</v>
+        <v>0.0536900847770649</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0365040756474625</v>
+        <v>0.0343616871945656</v>
       </c>
       <c r="Q2" t="n">
         <v>2008</v>
@@ -598,7 +598,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>750.442270032444</v>
+        <v>846.9368708602736</v>
       </c>
     </row>
     <row r="3">
@@ -616,35 +616,35 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.057580713001987</v>
+        <v>0.0478141755185989</v>
       </c>
       <c r="E3" t="n">
-        <v>5.758071300198706</v>
+        <v>4.781417551859893</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0358255433102198</v>
+        <v>0.0323836704553171</v>
       </c>
       <c r="G3" t="n">
-        <v>3.582554331021983</v>
+        <v>3.23836704553171</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1079988735443715</v>
+        <v>0.1398123155722116</v>
       </c>
       <c r="I3" t="n">
-        <v>-1.263606161262367</v>
+        <v>-1.56566522610364</v>
       </c>
       <c r="J3" t="n">
-        <v>12.77974876165978</v>
+        <v>11.12850032982343</v>
       </c>
       <c r="K3" t="n">
-        <v>934</v>
+        <v>689</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0978023117515803</v>
+        <v>0.1630276505269368</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>weight_t</t>
+          <t>earnwt_t</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -653,10 +653,10 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>0.057580713001987</v>
+        <v>0.0478141755185989</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0358255433102198</v>
+        <v>0.0323836704553171</v>
       </c>
       <c r="Q3" t="n">
         <v>2009</v>
@@ -668,7 +668,7 @@
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>779.1380771709728</v>
+        <v>953.5596318592965</v>
       </c>
     </row>
     <row r="4">
@@ -686,35 +686,35 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.0038520041475052</v>
+        <v>0.0636626972079065</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3852004147505225</v>
+        <v>6.366269720790658</v>
       </c>
       <c r="F4" t="n">
-        <v>0.037254357981069</v>
+        <v>0.0332096225045517</v>
       </c>
       <c r="G4" t="n">
-        <v>3.725435798106908</v>
+        <v>3.320962250455171</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9176475672026848</v>
+        <v>0.0552385021557944</v>
       </c>
       <c r="I4" t="n">
-        <v>-6.916519576255249</v>
+        <v>-0.1426966841185623</v>
       </c>
       <c r="J4" t="n">
-        <v>7.686920405756294</v>
+        <v>12.87523612569988</v>
       </c>
       <c r="K4" t="n">
-        <v>866</v>
+        <v>645</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1256685618289303</v>
+        <v>0.2760742112635699</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>weight_t</t>
+          <t>earnwt_t</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -723,10 +723,10 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>0.0038520041475052</v>
+        <v>0.0636626972079065</v>
       </c>
       <c r="P4" t="n">
-        <v>0.037254357981069</v>
+        <v>0.0332096225045517</v>
       </c>
       <c r="Q4" t="n">
         <v>2010</v>
@@ -738,7 +738,7 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>720.5196562279364</v>
+        <v>906.7177592591598</v>
       </c>
     </row>
     <row r="5">
@@ -756,35 +756,35 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.0011884041551297</v>
+        <v>0.0284394392714213</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1188404155129715</v>
+        <v>2.843943927142132</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0385985218198338</v>
+        <v>0.0352464564225052</v>
       </c>
       <c r="G5" t="n">
-        <v>3.85985218198339</v>
+        <v>3.524645642250521</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9754379314474416</v>
+        <v>0.4197392432709966</v>
       </c>
       <c r="I5" t="n">
-        <v>-7.446330846822812</v>
+        <v>-4.064234589934937</v>
       </c>
       <c r="J5" t="n">
-        <v>7.684011677848757</v>
+        <v>9.752122444219202</v>
       </c>
       <c r="K5" t="n">
-        <v>803</v>
+        <v>593</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1246146345506944</v>
+        <v>0.2482346265518156</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>weight_t</t>
+          <t>earnwt_t</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -793,10 +793,10 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>0.0011884041551297</v>
+        <v>0.0284394392714213</v>
       </c>
       <c r="P5" t="n">
-        <v>0.0385985218198338</v>
+        <v>0.0352464564225052</v>
       </c>
       <c r="Q5" t="n">
         <v>2011</v>
@@ -808,7 +808,7 @@
         <v>1</v>
       </c>
       <c r="T5" t="n">
-        <v>671.2103640672381</v>
+        <v>804.9503219060355</v>
       </c>
     </row>
     <row r="6">
@@ -826,35 +826,35 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.0358328185338779</v>
+        <v>0.06360139556153691</v>
       </c>
       <c r="E6" t="n">
-        <v>3.583281853387796</v>
+        <v>6.360139556153698</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0388541875964546</v>
+        <v>0.0349565148022213</v>
       </c>
       <c r="G6" t="n">
-        <v>3.885418759645464</v>
+        <v>3.495651480222135</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3564043080010644</v>
+        <v>0.0688438305101076</v>
       </c>
       <c r="I6" t="n">
-        <v>-4.031998980373602</v>
+        <v>-0.4912114475858153</v>
       </c>
       <c r="J6" t="n">
-        <v>11.19856268714919</v>
+        <v>13.21149055989321</v>
       </c>
       <c r="K6" t="n">
-        <v>754</v>
+        <v>584</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1275029684660567</v>
+        <v>0.2306554469281969</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>weight_t</t>
+          <t>earnwt_t</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -863,10 +863,10 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>0.0358328185338779</v>
+        <v>0.06360139556153691</v>
       </c>
       <c r="P6" t="n">
-        <v>0.0388541875964546</v>
+        <v>0.0349565148022213</v>
       </c>
       <c r="Q6" t="n">
         <v>2012</v>
@@ -878,7 +878,7 @@
         <v>1</v>
       </c>
       <c r="T6" t="n">
-        <v>662.4061174263508</v>
+        <v>818.3587812704634</v>
       </c>
     </row>
     <row r="7">
@@ -896,35 +896,35 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.06834363735005</v>
+        <v>0.0488630321976003</v>
       </c>
       <c r="E7" t="n">
-        <v>6.834363735005009</v>
+        <v>4.886303219760038</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0392010253785429</v>
+        <v>0.0388737354390049</v>
       </c>
       <c r="G7" t="n">
-        <v>3.920102537854291</v>
+        <v>3.887373543900496</v>
       </c>
       <c r="H7" t="n">
-        <v>0.08126123154427931</v>
+        <v>0.2087653097725085</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.8488960548934665</v>
+        <v>-2.732808920738769</v>
       </c>
       <c r="J7" t="n">
-        <v>14.51762352490348</v>
+        <v>12.50541536025885</v>
       </c>
       <c r="K7" t="n">
-        <v>660</v>
+        <v>562</v>
       </c>
       <c r="L7" t="n">
-        <v>0.2531075173843791</v>
+        <v>0.2706871679615602</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>weight_t</t>
+          <t>earnwt_t</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -933,10 +933,10 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>0.06834363735005</v>
+        <v>0.0488630321976003</v>
       </c>
       <c r="P7" t="n">
-        <v>0.0392010253785429</v>
+        <v>0.0388737354390049</v>
       </c>
       <c r="Q7" t="n">
         <v>2013</v>
@@ -948,7 +948,7 @@
         <v>1</v>
       </c>
       <c r="T7" t="n">
-        <v>650.7364684121268</v>
+        <v>661.7400967979514</v>
       </c>
     </row>
     <row r="8">
@@ -966,35 +966,35 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>-0.0202441064424164</v>
+        <v>-0.0216292251698924</v>
       </c>
       <c r="E8" t="n">
-        <v>-2.024410644241641</v>
+        <v>-2.162922516989247</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0380662266964344</v>
+        <v>0.0381107258048094</v>
       </c>
       <c r="G8" t="n">
-        <v>3.806622669643449</v>
+        <v>3.811072580480942</v>
       </c>
       <c r="H8" t="n">
-        <v>0.5948556595442202</v>
+        <v>0.5703497848436563</v>
       </c>
       <c r="I8" t="n">
-        <v>-9.485253979476512</v>
+        <v>-9.632487517200021</v>
       </c>
       <c r="J8" t="n">
-        <v>5.436432690993231</v>
+        <v>5.306642483221525</v>
       </c>
       <c r="K8" t="n">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="L8" t="n">
-        <v>0.2779386571290255</v>
+        <v>0.2702953784260596</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>weight_t</t>
+          <t>earnwt_t</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1003,10 +1003,10 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>-0.0202441064424164</v>
+        <v>-0.0216292251698924</v>
       </c>
       <c r="P8" t="n">
-        <v>0.0380662266964344</v>
+        <v>0.0381107258048094</v>
       </c>
       <c r="Q8" t="n">
         <v>2014</v>
@@ -1018,7 +1018,7 @@
         <v>1</v>
       </c>
       <c r="T8" t="n">
-        <v>690.1132101156807</v>
+        <v>688.5025614961115</v>
       </c>
     </row>
     <row r="9">
@@ -1036,35 +1036,35 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>-0.07321379877547909</v>
+        <v>-0.0751774774795199</v>
       </c>
       <c r="E9" t="n">
-        <v>-7.321379877547914</v>
+        <v>-7.517747747951997</v>
       </c>
       <c r="F9" t="n">
-        <v>0.039753144295954</v>
+        <v>0.0399038563489977</v>
       </c>
       <c r="G9" t="n">
-        <v>3.975314429595405</v>
+        <v>3.990385634899773</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0655174503769113</v>
+        <v>0.0595696802282353</v>
       </c>
       <c r="I9" t="n">
-        <v>-15.1128529867773</v>
+        <v>-15.33875987678155</v>
       </c>
       <c r="J9" t="n">
-        <v>0.470093231681469</v>
+        <v>0.3032643808775562</v>
       </c>
       <c r="K9" t="n">
-        <v>568</v>
+        <v>556</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2816594851022083</v>
+        <v>0.2877110124607603</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>weight_t</t>
+          <t>earnwt_t</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1073,10 +1073,10 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>-0.07321379877547909</v>
+        <v>-0.0751774774795199</v>
       </c>
       <c r="P9" t="n">
-        <v>0.039753144295954</v>
+        <v>0.0399038563489977</v>
       </c>
       <c r="Q9" t="n">
         <v>2015</v>
@@ -1088,7 +1088,7 @@
         <v>1</v>
       </c>
       <c r="T9" t="n">
-        <v>632.7862443411478</v>
+        <v>628.0153562594587</v>
       </c>
     </row>
     <row r="10">
@@ -1106,35 +1106,35 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>-0.0107420481461916</v>
+        <v>-0.0235225341739675</v>
       </c>
       <c r="E10" t="n">
-        <v>-1.074204814619161</v>
+        <v>-2.35225341739675</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0413986868272394</v>
+        <v>0.0414623053393251</v>
       </c>
       <c r="G10" t="n">
-        <v>4.13986868272394</v>
+        <v>4.146230533932515</v>
       </c>
       <c r="H10" t="n">
-        <v>0.7952664601992031</v>
+        <v>0.5704945122654734</v>
       </c>
       <c r="I10" t="n">
-        <v>-9.18819833348336</v>
+        <v>-10.47871593550476</v>
       </c>
       <c r="J10" t="n">
-        <v>7.03978870424504</v>
+        <v>5.774209100711257</v>
       </c>
       <c r="K10" t="n">
-        <v>529</v>
+        <v>518</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2488592752312309</v>
+        <v>0.2558967096173768</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>weight_t</t>
+          <t>earnwt_t</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1143,10 +1143,10 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>-0.0107420481461916</v>
+        <v>-0.0235225341739675</v>
       </c>
       <c r="P10" t="n">
-        <v>0.0413986868272394</v>
+        <v>0.0414623053393251</v>
       </c>
       <c r="Q10" t="n">
         <v>2016</v>
@@ -1158,7 +1158,7 @@
         <v>1</v>
       </c>
       <c r="T10" t="n">
-        <v>583.4812021961156</v>
+        <v>581.6920239269692</v>
       </c>
     </row>
   </sheetData>
@@ -1219,19 +1219,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.287</v>
+        <v>5.496</v>
       </c>
       <c r="C2" t="n">
-        <v>2.353</v>
+        <v>2.253</v>
       </c>
       <c r="D2" t="n">
-        <v>0.205</v>
+        <v>0.0448</v>
       </c>
       <c r="E2" t="n">
-        <v>-2.276</v>
+        <v>0.169</v>
       </c>
       <c r="F2" t="n">
-        <v>8.85</v>
+        <v>10.823</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -1246,19 +1246,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-3.224</v>
+        <v>-4.743</v>
       </c>
       <c r="C3" t="n">
-        <v>2.956</v>
+        <v>2.891</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3114</v>
+        <v>0.1449</v>
       </c>
       <c r="E3" t="n">
-        <v>-10.213</v>
+        <v>-11.58</v>
       </c>
       <c r="F3" t="n">
-        <v>3.764</v>
+        <v>2.093</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>

</xml_diff>